<commit_message>
feat: add editable files
</commit_message>
<xml_diff>
--- a/manuals/QUALITY MANUAL (QM) Ver2/Forms/QM Forms (editable copy)/PSHS-00-F-QMS-01-Ver02-Rev0 Document Change Request.xlsx
+++ b/manuals/QUALITY MANUAL (QM) Ver2/Forms/QM Forms (editable copy)/PSHS-00-F-QMS-01-Ver02-Rev0 Document Change Request.xlsx
@@ -1,23 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11700"/>
-  </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr/>
   <extLst>
-    <ext uri="GoogleSheetsCustomDataVersion1">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataSignature="AMtx7mjcK/yMCj5rwkBZIJj+Lgm6DK3Rgw=="/>
+    <ext uri="GoogleSheetsCustomDataVersion2">
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="3SJ90WeKKgbP+lFnS3gQYO2D1rsFVt8M7MxCJ1Q9GCM="/>
     </ext>
   </extLst>
 </workbook>
@@ -32,55 +24,163 @@
     <t>DOCUMENT CHANGE REQUEST</t>
   </si>
   <si>
+    <t>DATE :  ___________________                                                DCR No.  _________</t>
+  </si>
+  <si>
+    <t>TO     :  _______________________</t>
+  </si>
+  <si>
+    <t>FROM : ____________________</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amend document  [   ]  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">New document  [   ]  </t>
+  </si>
+  <si>
     <t>Delete document  [   ]</t>
   </si>
   <si>
     <t xml:space="preserve">1. DETAILS OF DOCUMENT </t>
-  </si>
-  <si>
-    <t>Note:  Please attach draft copy of the document.</t>
-  </si>
-  <si>
-    <t>2. CHANGE(S) REQUESTED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REASON FOR THE CHANGE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">     </t>
-  </si>
-  <si>
-    <t>Requested by</t>
-  </si>
-  <si>
-    <t>Reviewed by (Division Chief)</t>
-  </si>
-  <si>
-    <t>3. QMR’S COMMENTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">                                                                                                                                    Signature/Date</t>
-  </si>
-  <si>
-    <t>4. RECOMMENDING APPROVAL</t>
   </si>
   <si>
     <r>
       <rPr>
-        <sz val="8"/>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>Document Number</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t xml:space="preserve"> : ______________________________________</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>Document Title</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t xml:space="preserve"> : ______________________________________</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>Revision Status</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t xml:space="preserve"> : _____________________________________</t>
+    </r>
+  </si>
+  <si>
+    <t>Note:  Please attach draft copy of the document.</t>
+  </si>
+  <si>
+    <t>2. CHANGE(S) REQUESTED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REASON FOR THE CHANGE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">     </t>
+  </si>
+  <si>
+    <t>Requested by</t>
+  </si>
+  <si>
+    <t>Reviewed by (Division Chief)</t>
+  </si>
+  <si>
+    <t>3. QMR’S COMMENTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t xml:space="preserve">    Request Denied  [   ]                    Request Accepted  [   ]</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t xml:space="preserve">                          _________________________</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">                                                                                                                                    Signature/Date</t>
+  </si>
+  <si>
+    <t>4. RECOMMENDING APPROVAL</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t xml:space="preserve">5. </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>APPROVING AUTHORITY</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
         <color rgb="FF000000"/>
-        <rFont val="Arial"/>
+        <sz val="8.0"/>
       </rPr>
       <t xml:space="preserve">   </t>
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
+        <rFont val="Arial"/>
         <color rgb="FF000000"/>
-        <rFont val="Arial"/>
+        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">       Signature over printed name                 Date        </t>
     </r>
@@ -93,183 +193,102 @@
   </si>
   <si>
     <t>New Document Status        No.: ________  Version: ________ Revision: ________</t>
-  </si>
-  <si>
-    <t>DATE :  ___________________                                                DCR No.  _________</t>
-  </si>
-  <si>
-    <t>TO     :  _______________________</t>
-  </si>
-  <si>
-    <t>FROM : ____________________</t>
-  </si>
-  <si>
-    <r>
-      <t>Document Number</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve"> : ______________________________________</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Document Title</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve"> : ______________________________________</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Revision Status</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve"> : _____________________________________</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">New document  [   ]  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amend document  [   ]  </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">    Request Denied  [   ]                    Request Accepted  [   ]</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">                          _________________________</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">5. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>APPROVING AUTHORITY</t>
-    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="17">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <fonts count="18">
     <font>
-      <sz val="11"/>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="12.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font/>
+    <font>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="6.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="6"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8"/>
+      <sz val="8.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="4"/>
+      <sz val="4.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="3"/>
+      <sz val="3.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="8.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="5"/>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="5.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -279,228 +298,181 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="lightGray"/>
     </fill>
   </fills>
   <borders count="9">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
     <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
-      <right/>
       <top style="medium">
         <color rgb="FF000000"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
       <top style="medium">
         <color rgb="FF000000"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
       <top style="medium">
         <color rgb="FF000000"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
-      <right/>
-      <top/>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
-      <top/>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="41">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="37">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -690,516 +662,365 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z997"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <pageSetUpPr/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
-    <col min="3" max="3" width="6.85546875" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="6" width="13.85546875" customWidth="1"/>
-    <col min="7" max="7" width="18.140625" customWidth="1"/>
-    <col min="8" max="26" width="8.7109375" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="16.86"/>
+    <col customWidth="1" min="2" max="2" width="19.57"/>
+    <col customWidth="1" min="3" max="3" width="6.86"/>
+    <col customWidth="1" min="4" max="4" width="15.0"/>
+    <col customWidth="1" min="5" max="6" width="13.86"/>
+    <col customWidth="1" min="7" max="7" width="18.14"/>
+    <col customWidth="1" min="8" max="26" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A1" s="38" t="s">
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="11"/>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="39" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="17"/>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="40"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="11"/>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1">
-      <c r="A4" s="34" t="s">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="6"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" ht="30.0" customHeight="1">
+      <c r="A4" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="9"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="10"/>
+      <c r="G5" s="9"/>
+    </row>
+    <row r="6" ht="15.0" customHeight="1">
+      <c r="A6" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="9"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10"/>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" ht="21.75" customHeight="1">
+      <c r="A8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G8" s="9"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="3"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="13"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="15"/>
+    </row>
+    <row r="11" ht="15.0" customHeight="1">
+      <c r="A11" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="17"/>
+      <c r="G12" s="9"/>
+    </row>
+    <row r="13" ht="25.5" customHeight="1">
+      <c r="A13" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" ht="25.5" customHeight="1">
+      <c r="A14" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="9"/>
+    </row>
+    <row r="15" ht="25.5" customHeight="1">
+      <c r="A15" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" ht="25.5" customHeight="1">
+      <c r="A16" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" ht="15.0" customHeight="1">
+      <c r="A17" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="3"/>
+    </row>
+    <row r="18" ht="18.75" customHeight="1">
+      <c r="A18" s="17"/>
+      <c r="G18" s="9"/>
+    </row>
+    <row r="19" ht="18.75" customHeight="1">
+      <c r="A19" s="17"/>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" ht="18.75" customHeight="1">
+      <c r="A20" s="17"/>
+      <c r="G20" s="9"/>
+    </row>
+    <row r="21" ht="18.75" customHeight="1">
+      <c r="A21" s="17"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" ht="18.75" customHeight="1">
+      <c r="A22" s="21"/>
+      <c r="G22" s="9"/>
+    </row>
+    <row r="23" ht="15.0" customHeight="1">
+      <c r="A23" s="22"/>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" ht="15.0" customHeight="1">
+      <c r="A24" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" s="9"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="17"/>
+      <c r="G26" s="9"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="17"/>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="23"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24"/>
+      <c r="N28" s="24"/>
+      <c r="O28" s="24"/>
+      <c r="P28" s="24"/>
+      <c r="Q28" s="24"/>
+      <c r="R28" s="24"/>
+      <c r="S28" s="24"/>
+      <c r="T28" s="24"/>
+      <c r="U28" s="24"/>
+      <c r="V28" s="24"/>
+      <c r="W28" s="24"/>
+      <c r="X28" s="24"/>
+      <c r="Y28" s="24"/>
+      <c r="Z28" s="24"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="17"/>
+      <c r="B29" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="F29" s="25"/>
+      <c r="G29" s="27"/>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="28"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="6"/>
+    </row>
+    <row r="31" ht="15.0" customHeight="1">
+      <c r="A31" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="14"/>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="35"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="14"/>
-    </row>
-    <row r="6" spans="1:7" ht="15" customHeight="1">
-      <c r="A6" s="34" t="s">
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="3"/>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="14"/>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="35"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="14"/>
-    </row>
-    <row r="8" spans="1:7" ht="21.75" customHeight="1">
-      <c r="A8" s="34" t="s">
+      <c r="G32" s="9"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="18"/>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="18"/>
+      <c r="G34" s="9"/>
+    </row>
+    <row r="35" ht="28.5" customHeight="1">
+      <c r="A35" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="14"/>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="36" t="s">
+      <c r="G35" s="9"/>
+    </row>
+    <row r="36" ht="25.5" customHeight="1">
+      <c r="A36" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="9"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="29"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="6"/>
+    </row>
+    <row r="38" ht="30.0" customHeight="1">
+      <c r="A38" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" s="2"/>
+      <c r="G38" s="3"/>
+    </row>
+    <row r="39" ht="30.75" customHeight="1">
+      <c r="A39" s="31"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="32"/>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" ht="24.0" customHeight="1">
+      <c r="A40" s="33" t="s">
+        <v>24</v>
+      </c>
+      <c r="D40" s="9"/>
+      <c r="E40" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="37" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="37" t="s">
-        <v>2</v>
-      </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="11"/>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="1"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="3"/>
-    </row>
-    <row r="11" spans="1:7" ht="15" customHeight="1">
-      <c r="A11" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="14"/>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="18"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="14"/>
-    </row>
-    <row r="13" spans="1:7" ht="25.5" customHeight="1">
-      <c r="A13" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="14"/>
-    </row>
-    <row r="14" spans="1:7" ht="25.5" customHeight="1">
-      <c r="A14" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="14"/>
-    </row>
-    <row r="15" spans="1:7" ht="25.5" customHeight="1">
-      <c r="A15" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="14"/>
-    </row>
-    <row r="16" spans="1:7" ht="25.5" customHeight="1">
-      <c r="A16" s="32" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="17"/>
-    </row>
-    <row r="17" spans="1:26" ht="15" customHeight="1">
-      <c r="A17" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="11"/>
-    </row>
-    <row r="18" spans="1:26" ht="18.75" customHeight="1">
-      <c r="A18" s="18"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="14"/>
-    </row>
-    <row r="19" spans="1:26" ht="18.75" customHeight="1">
-      <c r="A19" s="18"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="14"/>
-    </row>
-    <row r="20" spans="1:26" ht="18.75" customHeight="1">
-      <c r="A20" s="18"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="14"/>
-    </row>
-    <row r="21" spans="1:26" ht="18.75" customHeight="1">
-      <c r="A21" s="18"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="14"/>
-    </row>
-    <row r="22" spans="1:26" ht="18.75" customHeight="1">
-      <c r="A22" s="30"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="14"/>
-    </row>
-    <row r="23" spans="1:26" ht="15" customHeight="1">
-      <c r="A23" s="27"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="14"/>
-    </row>
-    <row r="24" spans="1:26" ht="15" customHeight="1">
-      <c r="A24" s="31" t="s">
-        <v>6</v>
-      </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="14"/>
-    </row>
-    <row r="25" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A25" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="14"/>
-    </row>
-    <row r="26" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A26" s="18"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="14"/>
-    </row>
-    <row r="27" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A27" s="18"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="14"/>
-    </row>
-    <row r="28" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A28" s="28"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
-      <c r="L28" s="5"/>
-      <c r="M28" s="5"/>
-      <c r="N28" s="5"/>
-      <c r="O28" s="5"/>
-      <c r="P28" s="5"/>
-      <c r="Q28" s="5"/>
-      <c r="R28" s="5"/>
-      <c r="S28" s="5"/>
-      <c r="T28" s="5"/>
-      <c r="U28" s="5"/>
-      <c r="V28" s="5"/>
-      <c r="W28" s="5"/>
-      <c r="X28" s="5"/>
-      <c r="Y28" s="5"/>
-      <c r="Z28" s="5"/>
-    </row>
-    <row r="29" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A29" s="4"/>
-      <c r="B29" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F29" s="6"/>
-      <c r="G29" s="8"/>
-    </row>
-    <row r="30" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A30" s="29"/>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="17"/>
-    </row>
-    <row r="31" spans="1:26" ht="15" customHeight="1">
-      <c r="A31" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="11"/>
-    </row>
-    <row r="32" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A32" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="14"/>
-    </row>
-    <row r="33" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A33" s="12"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="14"/>
-    </row>
-    <row r="34" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A34" s="12"/>
-      <c r="B34" s="13"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="14"/>
-    </row>
-    <row r="35" spans="1:7" ht="28.5" customHeight="1">
-      <c r="A35" s="12" t="s">
+      <c r="G40" s="9"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="35"/>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="36"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="6"/>
+    </row>
+    <row r="42" ht="15.0" customHeight="1">
+      <c r="A42" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="B35" s="13"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="14"/>
-    </row>
-    <row r="36" spans="1:7" ht="25.5" customHeight="1">
-      <c r="A36" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="14"/>
-    </row>
-    <row r="37" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A37" s="19"/>
-      <c r="B37" s="16"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="17"/>
-    </row>
-    <row r="38" spans="1:7" ht="30" customHeight="1">
-      <c r="A38" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="20" t="s">
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="3"/>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="18"/>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="A44" s="18"/>
+      <c r="G44" s="9"/>
+    </row>
+    <row r="45" ht="28.5" customHeight="1">
+      <c r="A45" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="F38" s="10"/>
-      <c r="G38" s="11"/>
-    </row>
-    <row r="39" spans="1:7" ht="30.75" customHeight="1">
-      <c r="A39" s="22"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="23"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="14"/>
-    </row>
-    <row r="40" spans="1:7" ht="24" customHeight="1">
-      <c r="A40" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="F40" s="13"/>
-      <c r="G40" s="14"/>
-    </row>
-    <row r="41" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A41" s="21"/>
-      <c r="B41" s="16"/>
-      <c r="C41" s="16"/>
-      <c r="D41" s="17"/>
-      <c r="E41" s="26"/>
-      <c r="F41" s="16"/>
-      <c r="G41" s="17"/>
-    </row>
-    <row r="42" spans="1:7" ht="15" customHeight="1">
-      <c r="A42" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="10"/>
-      <c r="G42" s="11"/>
-    </row>
-    <row r="43" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A43" s="12"/>
-      <c r="B43" s="13"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="14"/>
-    </row>
-    <row r="44" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A44" s="12"/>
-      <c r="B44" s="13"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="14"/>
-    </row>
-    <row r="45" spans="1:7" ht="28.5" customHeight="1">
-      <c r="A45" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B45" s="13"/>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="14"/>
-    </row>
-    <row r="46" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A46" s="15"/>
-      <c r="B46" s="16"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="16"/>
-      <c r="F46" s="16"/>
-      <c r="G46" s="17"/>
-    </row>
-    <row r="47" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="48" spans="1:7" ht="15.75" customHeight="1"/>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="13"/>
+      <c r="B46" s="5"/>
+      <c r="C46" s="5"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="6"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1"/>
+    <row r="48" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>
@@ -2175,10 +1996,10 @@
     <mergeCell ref="A20:G20"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A23:G23"/>
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A25:G25"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A23:G23"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A28:G28"/>
     <mergeCell ref="A30:G30"/>
@@ -2191,22 +2012,24 @@
     <mergeCell ref="A37:G37"/>
     <mergeCell ref="A38:D38"/>
     <mergeCell ref="E38:G38"/>
-    <mergeCell ref="A41:D41"/>
     <mergeCell ref="A39:D39"/>
     <mergeCell ref="E39:G39"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A46:G46"/>
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="E40:G40"/>
+    <mergeCell ref="A41:D41"/>
     <mergeCell ref="E41:G41"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A44:G44"/>
-    <mergeCell ref="A45:G45"/>
-    <mergeCell ref="A46:G46"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="84" orientation="portrait" r:id="rId1"/>
+  <printOptions/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup paperSize="9" scale="84" orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;LPSHS-00-F-QMS-01-Ver02-Rev0-02/01/20</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>